<commit_message>
can runs step by step but without updating mass flow rate and temperature
</commit_message>
<xml_diff>
--- a/GeoInput.xlsx
+++ b/GeoInput.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\08-ParallelSyncBoreholes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\trnsys-bns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F564E678-5FEB-4BC1-9C31-8E28E3664A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646A2A2E-05CB-4C0F-A200-292850FC0360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Borehole" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>H [m]</t>
   </si>
@@ -77,9 +77,6 @@
     <t>870.0</t>
   </si>
   <si>
-    <t>0.1</t>
-  </si>
-  <si>
     <t>Rb [mK/W]</t>
   </si>
   <si>
@@ -87,6 +84,9 @@
   </si>
   <si>
     <t>cp [J/(kgK)]</t>
+  </si>
+  <si>
+    <t>activation_year</t>
   </si>
 </sst>
 </file>
@@ -410,13 +410,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="5" width="8.7265625" style="1"/>
+    <col min="6" max="6" width="13.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,8 +434,11 @@
       <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>100</v>
       </c>
@@ -449,8 +454,11 @@
       <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>100</v>
       </c>
@@ -460,11 +468,54 @@
       <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>13</v>
+      <c r="D3" s="2">
+        <v>1</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>100</v>
+      </c>
+      <c r="B4" s="2">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>100</v>
+      </c>
+      <c r="B5" s="2">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -495,10 +546,10 @@
         <v>10</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -534,7 +585,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
simulations work with old methods, need to clean
</commit_message>
<xml_diff>
--- a/GeoInput.xlsx
+++ b/GeoInput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\trnsys-bns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646A2A2E-05CB-4C0F-A200-292850FC0360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16631C1A-062E-4470-8997-DD09C68771DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Borehole" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>H [m]</t>
   </si>
@@ -410,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="5" width="8.7265625" style="1"/>
@@ -440,7 +443,7 @@
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="B2" s="2">
         <v>6</v>
@@ -458,9 +461,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="B3" s="2">
         <v>6</v>
@@ -469,18 +472,18 @@
         <v>3</v>
       </c>
       <c r="D3" s="2">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="B4" s="2">
         <v>6</v>
@@ -492,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="1">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F4" s="1">
         <v>3</v>
@@ -500,7 +503,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="B5" s="2">
         <v>6</v>
@@ -509,14 +512,44 @@
         <v>3</v>
       </c>
       <c r="D5" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" s="1">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="F5" s="1">
         <v>3</v>
       </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
tests running, some cleaning
</commit_message>
<xml_diff>
--- a/GeoInput.xlsx
+++ b/GeoInput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\trnsys-bns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16631C1A-062E-4470-8997-DD09C68771DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE19ABC-2F23-4D80-A206-5EE7032B17A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Borehole" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>H [m]</t>
   </si>
@@ -86,10 +86,22 @@
     <t>Tg [degC]</t>
   </si>
   <si>
-    <t>cp [J/(kgK)]</t>
-  </si>
-  <si>
     <t>activation_year</t>
+  </si>
+  <si>
+    <t>Select Fluid</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Fluids Explanation</t>
+  </si>
+  <si>
+    <t>EthanolMix: 20% ethanol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GlycolMix: 30% glycol </t>
   </si>
 </sst>
 </file>
@@ -113,7 +125,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -121,11 +133,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -133,6 +184,9 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,7 +492,7 @@
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -610,23 +664,40 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B04DB288-D233-43AD-80D6-9BAE58C6DDCA}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.1796875" customWidth="1"/>
+    <col min="3" max="3" width="21.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>4217</v>
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{CA38D562-456F-480B-8A1A-3E5824712529}">
+      <formula1>"Water,EthanolMix,GlycolMix"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added dependency on fork
</commit_message>
<xml_diff>
--- a/GeoInput.xlsx
+++ b/GeoInput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\trnsys-bns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE19ABC-2F23-4D80-A206-5EE7032B17A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C5B6E4-EC19-4B6D-8449-CB8C77F71E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Borehole" sheetId="1" r:id="rId1"/>
@@ -557,7 +557,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B5" s="2">
         <v>6</v>

</xml_diff>

<commit_message>
fixed bug with Q2 calculation
</commit_message>
<xml_diff>
--- a/GeoInput.xlsx
+++ b/GeoInput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\trnsys-bns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82AC50C-BE56-4306-8E5C-BF93A438D3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F0D199-E04C-49B6-9B26-80CE0788EFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Borehole" sheetId="1" r:id="rId1"/>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="5" width="8.7265625" style="1"/>
@@ -514,7 +514,7 @@
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="B3" s="2">
         <v>6</v>
@@ -522,17 +522,17 @@
       <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
         <v>3</v>
       </c>
-      <c r="E3" s="2">
-        <v>0</v>
-      </c>
       <c r="F3" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>150</v>
       </c>
@@ -543,13 +543,13 @@
         <v>3</v>
       </c>
       <c r="D4" s="1">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1">
         <v>0</v>
       </c>
-      <c r="E4" s="1">
-        <v>3</v>
-      </c>
       <c r="F4" s="1">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -581,11 +581,6 @@
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>